<commit_message>
feat: implement backend service layer and agentic orchestration for the Utilities Knowledge Hub chatbot
</commit_message>
<xml_diff>
--- a/app/data/Knowledge_Base.xlsx
+++ b/app/data/Knowledge_Base.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,264 +441,682 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Worcester Bosch 4000</t>
+          <t>Centrica Enterprise Platform</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>displays_error</t>
+          <t>powers</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>EA_Error</t>
+          <t>Agentic Knowledge Hub</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Flame not detected after ignition attempt.</t>
+          <t>Unified AI-powered intelligence layer for Centrica business knowledge, datasets, dashboards, and operational insights.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EA_Error</t>
+          <t>Sales_Funnel_Dataset</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>requires_part</t>
+          <t>managed_by_sme</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Ignition Electrode</t>
+          <t>Sarah Jenkins (Head of Commercial Analytics)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Inspect lead connection, clean electrode or replace if worn.</t>
+          <t>Owner of commercial sales funnel, lead attribution, and conversion metrics in Snowflake.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EA_Error</t>
+          <t>Sales_Funnel_Dataset</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>requires_part</t>
+          <t>lineage_source</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Gas Supply Valve</t>
+          <t>SAP IS-U &amp; Salesforce CRM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Check gas inlet pressure and solenoid valve coil resistance.</t>
+          <t>Aggregates raw customer leads and survey appointments from Salesforce into Snowflake data lake.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EA_Error</t>
+          <t>Live_Metrics_Dataset</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>caused_by</t>
+          <t>managed_by_sme</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Low Gas Pressure</t>
+          <t>David Ross (Lead Telemetry Engineer)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Gas supply pressure at meter is below 18 mbar.</t>
+          <t>Maintains IoT grid pressure and thermal telemetry sensors across UK regions.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Low Gas Pressure</t>
+          <t>Live_Metrics_Dataset</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>remedy_step</t>
+          <t>lineage_source</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Check Emergency Control Valve</t>
+          <t>Grid Mon Substation IoT Network</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Ensure main ECV valve handle is aligned parallel to gas pipe.</t>
+          <t>Real-time telemetry ingested via Kafka into Snowflake Operational Data Store.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Worcester Bosch 4000</t>
+          <t>Boiler_Installation_Forecast_v2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>displays_error</t>
+          <t>managed_by_sme</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>224_Error</t>
+          <t>Marcus Vance (Principal Data Scientist)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Primary flue thermostat or safety limiter tripped (&gt;105°C).</t>
+          <t>Predictive installation model using pipeline conversion, seasonal demand, and engineer capacity.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>224_Error</t>
+          <t>Boiler_Installation_Forecast_v2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>caused_by</t>
+          <t>consumes_dataset</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Overheating</t>
+          <t>Sales_Funnel_Dataset</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>System water flow restricted or pump air locked.</t>
+          <t>Uses qualified lead volume, kept appointment ratios, and quote conversion rates.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Overheating</t>
+          <t>Centrica_Executive_Dashboard</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>requires_part</t>
+          <t>managed_by_sme</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Circulating Pump</t>
+          <t>Claire Williams (VP Operations)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Verify pump impeller spin and clear air bleed valve.</t>
+          <t>PowerBI dashboard providing real-time visibility into sales conversion, telemetry alerts, and service activity.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ideal Logic Combi</t>
+          <t>Centrica_Executive_Dashboard</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>displays_error</t>
+          <t>displays_metrics</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>F2_Error</t>
+          <t>Sales Conversion &amp; Grid Telemetry</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Flame loss during operation.</t>
+          <t>Unified view combining Commercial Sales Funnel and Live Telemetry Metrics.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>F2_Error</t>
+          <t>Worcester Bosch 4000</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>requires_part</t>
+          <t>displays_error</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Condensate Pipe</t>
+          <t>EA_Error</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Check for external ice blockage or kinked discharge pipe.</t>
+          <t>Flame was not detected after an ignition attempt.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Baxi 800 Combi</t>
+          <t>EA_Error</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>displays_error</t>
+          <t>requires_part</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>E119_Error</t>
+          <t>Ignition Electrode</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>System operating pressure below minimum threshold (&lt;0.5 bar).</t>
+          <t>Inspect the lead, clean the electrode, or replace it if worn.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>EA_Error</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>requires_part</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Gas Supply Valve</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Check inlet pressure and the solenoid valve coil resistance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>EA_Error</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>caused_by</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Low Gas Pressure</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Gas pressure at the meter is below 18 mbar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Low Gas Pressure</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>remedy_step</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Check Emergency Control Valve</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Ensure the main valve handle is parallel to the pipe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Worcester Bosch 4000</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>displays_error</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>224_Error</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>The primary flue thermostat or safety limiter has tripped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>224_Error</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>caused_by</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Overheating</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Water flow may be restricted or the pump may be air locked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Overheating</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>requires_part</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Circulating Pump</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Verify impeller movement and bleed trapped air.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ideal Logic Combi</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>displays_error</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>F2_Error</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Flame loss during operation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>F2_Error</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>requires_part</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Condensate Pipe</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Check for external ice blockage or a kinked discharge pipe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Baxi 800 Combi</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>displays_error</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>E119_Error</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>System pressure is below the minimum operating threshold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>E119_Error</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
         <is>
           <t>remedy_step</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Re-pressurise Filling Loop</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Attach filling loop hose and repressurise system gauge to 1.5 bar.</t>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Repressurise the system gauge to 1.5 bar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Home Energy Services</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>provides</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Heating Installation</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Design and fit replacement boilers, heating controls, and compatible system upgrades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Home Energy Services</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>provides</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Heating Repair</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Diagnose and repair boiler, radiator, thermostat, and hot-water faults.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Home Energy Services</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>provides</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Annual Maintenance</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Carry out planned appliance servicing and safety checks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Home Energy Services</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>provides</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Plumbing And Drains</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Repair leaks, taps, toilets, pipework, and common drainage issues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Home Energy Services</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>provides</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Electrical Support</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Provide domestic electrical checks, fault diagnosis, and selected repairs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Home Energy Services</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>provides</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Appliance Care</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Repair and maintain selected kitchen and laundry appliances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>converts_to</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Net Appointment</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>A qualified prospect that results in a kept consultation or survey appointment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Net Appointment</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>converts_to</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Net Sale</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>A kept appointment that results in a completed, non-cancelled sale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Net Sale</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>measured_by</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Sales Conversion</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Net sales divided by qualified leads, expressed as a percentage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>supports</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Net Sale</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>A priced proposal issued for an installation, repair, or service plan.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement agentic chatbot architecture with RAG tools and deterministic fallback logic for dataset access and governance queries
</commit_message>
<xml_diff>
--- a/app/data/Knowledge_Base.xlsx
+++ b/app/data/Knowledge_Base.xlsx
@@ -441,7 +441,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Centrica Enterprise Platform</t>
+          <t>ABC Enterprise Platform</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -456,7 +456,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Unified AI-powered intelligence layer for Centrica business knowledge, datasets, dashboards, and operational insights.</t>
+          <t>Unified AI-powered intelligence layer for ABC business knowledge, datasets, dashboards, and operational insights.</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Centrica_Executive_Dashboard</t>
+          <t>ABC_Executive_Dashboard</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Centrica_Executive_Dashboard</t>
+          <t>ABC_Executive_Dashboard</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">

</xml_diff>

<commit_message>
feat: initialize Utilities Knowledge Hub project with Excel data sources and base services
</commit_message>
<xml_diff>
--- a/app/data/Knowledge_Base.xlsx
+++ b/app/data/Knowledge_Base.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1035,86 +1035,152 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Lead</t>
+          <t>EA_Error</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>converts_to</t>
+          <t>need_to_end_connection</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Net Appointment</t>
+          <t>Worcester Bosch 4000</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>A qualified prospect that results in a kept consultation or survey appointment.</t>
+          <t>Boiler must be isolated and power disconnected before any repair attempt — risk of electric shock and gas leak.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Net Appointment</t>
+          <t>224_Error</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>converts_to</t>
+          <t>need_to_end_connection</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Net Sale</t>
+          <t>Worcester Bosch 4000</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>A kept appointment that results in a completed, non-cancelled sale.</t>
+          <t>Overheating fault requires immediate shutdown and full system isolation before engineer intervention.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Net Sale</t>
+          <t>E119_Error</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>measured_by</t>
+          <t>need_to_end_connection</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Sales Conversion</t>
+          <t>Baxi 800 Combi</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Net sales divided by qualified leads, expressed as a percentage.</t>
+          <t>Low pressure fault — isolate system and depressurise before opening any filling loop connections.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>converts_to</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Net Appointment</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>A qualified prospect that results in a kept consultation or survey appointment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Net Appointment</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>converts_to</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Net Sale</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>A kept appointment that results in a completed, non-cancelled sale.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Net Sale</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>measured_by</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Sales Conversion</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Net sales divided by qualified leads, expressed as a percentage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Quote</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>supports</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Net Sale</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>A priced proposal issued for an installation, repair, or service plan.</t>
         </is>

</xml_diff>